<commit_message>
Rates 10/25/50; cleaner readable tables; label agreed/half/floor
</commit_message>
<xml_diff>
--- a/Dutch-Ruby-Comp-Claim.xlsx
+++ b/Dutch-Ruby-Comp-Claim.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,10 +43,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="4">
@@ -93,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,12 +99,15 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -487,13 +486,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -574,12 +573,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Gross (hours × rate)</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Less paid</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -601,7 +600,7 @@
         <v>1060</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>-350</v>
+        <v>350</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>710</v>
@@ -610,103 +609,39 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>$50/hr</t>
+          <t>$25/hr</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
         <v>106</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>5300</v>
+        <v>2650</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>-350</v>
+        <v>350</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>4950</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>$150/hr</t>
+          <t>$50/hr</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
         <v>106</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>15900</v>
+        <v>5300</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>-350</v>
+        <v>350</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>15550</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Floor variant (hrs=82)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>$10/hr</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n">
-        <v>82</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>820</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>-350</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>$50/hr</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n">
-        <v>82</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>4100</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>-350</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>3750</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>$150/hr</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="n">
-        <v>82</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>12300</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>-350</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>11950</v>
+        <v>4950</v>
       </c>
     </row>
   </sheetData>
@@ -768,14 +703,14 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
+          <t>@ $25</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
           <t>@ $50</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>@ $150</t>
-        </is>
-      </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Repos / sample work</t>
@@ -783,416 +718,416 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ru</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="G5" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G7" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="G8" s="14" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">ruby-trivia — untracked files on iono/games-production: dc3e01f Archive iono games production </t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H9" s="15" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>ruby-labs — Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="G11" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H11" s="15" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>2400</v>
-      </c>
-      <c r="H12" s="15" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — CI: use plain bun install (lockfile drifts across bun versions) + resync bun.loc</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="G13" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="G13" s="14" t="n">
-        <v>2400</v>
-      </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="G14" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="G14" s="14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia — Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcb</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="G15" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia, ruby-trivia-handbook — Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="G16" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing — Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel we</t>
         </is>
@@ -1211,14 +1146,14 @@
       <c r="D17" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E17" s="13" t="n">
         <v>1060</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F17" s="13" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G17" s="13" t="n">
         <v>5300</v>
-      </c>
-      <c r="G17" s="16" t="n">
-        <v>15900</v>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
     </row>
@@ -1247,70 +1182,70 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>• Trivia PWA — daily quiz, practice, friend challenges, leaderboards, streaks, ranks/badges, 4 languages, installable</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>• Live multiplayer — realtime WebSocket lobbies, matchmaking, graceful reconnect</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>• Backend &amp; API — Hono/Bun server, auth/registration, game logic, SQLite→MariaDB migration + SQL translation</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>• Web3 holder layer — Solana wallet connect, holder verification, perks (multiplier, holders-only leaderboard, cosmetics)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>• On-chain / contracts — contract suite, result-signer seam, token integration</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>• Telegram bot gateway — in-chat trivia, stateless solo play, /stats</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>• Production infra / DevOps — multi-container, nginx, MariaDB, deploy scripts, live incident response</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>• App-store repackaging — Capacitor + multi-store editions</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>• Token launch support &amp; ops — Solana/Pump.fun launch, splash/CA, coordination</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>• Educational variant — ruby-trivia-classroom</t>
         </is>
@@ -1366,2540 +1301,2540 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>2026-05-29 22:58</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ruby-labs	feat: sync latest marketing landing from ruby-trivia + i18n; purge bushleague</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n">
+      <c r="A5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 10:58</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Ship Ruby Trivia classroom hub with library-themed UI for bushleague.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:41</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Fix shelf book launches, clay UI, classroom sounds and haptics.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Mobile-first layout and full main-repo trivia parity.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Fix deploy script staging cleanup on Windows.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:47</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:49</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Fix GitHub Actions deploy SSH key and scp paths.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:51</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Fix CI deploy rsync when scp nests files under dist/.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:56</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Remove Class from header; rename nav to Lessons.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:00</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Boost clay depth and sounds; drop fake leaderboard names.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n">
+      <c r="A14" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:03</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Replace open Create with curated quiz sets; drop unsigned custom questions.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n">
+      <c r="A15" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:04</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Fix nav sounds: play on tab click inside user gesture.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:05</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Stop defaulting player name to Ruby; clear persisted Ruby names.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:07</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Block Ruby as player name; no anonymous leaderboard rows.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n">
+      <c r="A18" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:08</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Add preferred Ruby Trivia logo to header.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:10</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Omit unnamed players from scoreboards; document backend contract.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:12</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Put Trivia above Lessons in nav.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:14</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Remove duplicate hero logo; use downloaded sound files for cues.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>2026-06-17 22:12</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>2026-06-17 22:15</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Fix deploy script line endings and static upload cleanup.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n">
+      <c r="A24" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 17:15</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 17:28</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Restructure mobile nav around Games hub and add Odie's Car.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n">
+      <c r="A26" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 22:45</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Add Bush League clay dress kit and apply theme to app shell.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 14:33</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 14:34</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Add single-repo workflow doc after consolidating on ruby-high/ruby-trivia.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>index on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n">
+      <c r="A30" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>untracked files on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n">
+      <c r="A31" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e675af6ce46b	2026-06-25T04:50:33-04:00	dutchiono-ruby-trivia	feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n">
+      <c r="A32" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>Ignore TypeScript build info files.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n">
+      <c r="A33" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>2026-06-21 02:51</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n">
+      <c r="A34" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:23</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:27</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Add auth intent persistence and fix live room invite flow.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n">
+      <c r="A36" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:33</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Harden anotherone deploy: exclude server node_modules from upload.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:37</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>Fix unreadable theme-option buttons on clay cards in dark mode.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n">
+      <c r="A38" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 14:45</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>Add side dock rail, RUBYSQUARE header mark, and clay contrast fixes.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 21:22</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>Remove third-party studio branding and add session handoff doc.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="n">
+      <c r="A40" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 06:22</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>Document single-branch workflow; rename archive branch.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="n">
+      <c r="A41" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="n">
+      <c r="A42" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="n">
+      <c r="A43" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="13" t="n">
+      <c r="A44" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="n">
+      <c r="A45" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:22</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>Use MP3-only sensory assets from Audacity exports.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="n">
+      <c r="A46" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:29</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>Add on-chain scaffold, chain signer API, brand assets, and trivia data.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="n">
+      <c r="A47" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:40</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>Show Ruby Trivia logo in minimized mobile header chrome.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="n">
+      <c r="A48" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 12:09</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>Fix minimized mobile header: slim RUBYSQUARE pill, no side rail.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="n">
+      <c r="A49" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 12:29</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Route nav sounds: zipper on top dock, page on bottom subnav, paper on ranks.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="n">
+      <c r="A50" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 15:56</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>Refactor trivia navigation: bottom nav, mode nav, games layout</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="n">
+      <c r="A51" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 18:26</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>Fix unreadable secondary buttons on cream modals</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="n">
+      <c r="A52" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 19:46</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>Fix missing desktop nav rail in authenticated layout</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="n">
+      <c r="A53" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="13" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:02</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D53" s="15" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>Warm blue chrome to clay palette + add Docs to desktop nav</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="n">
+      <c r="A54" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:07</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D54" s="15" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>Reskin splash CTA from blue to clay orange</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="n">
+      <c r="A55" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:09</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D55" s="15" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>Warm active language-picker chip to clay orange</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="n">
+      <c r="A56" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B56" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:12</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D56" s="15" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>Warm language-button focus outline to clay orange</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="n">
+      <c r="A57" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B57" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:34</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>Public /docs route, clay answer buttons, warm crew links</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="n">
+      <c r="A58" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="B58" s="13" t="inlineStr">
+      <c r="B58" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:43</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>Fix production DB corruption: stop deploy from clobbering the live SQLite db</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="n">
+      <c r="A59" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B59" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:06</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>Add PR CI: build + chain tests</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="n">
+      <c r="A60" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="13" t="inlineStr">
+      <c r="B60" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:08</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>CI: use plain bun install (lockfile drifts across bun versions) + resync bun.lock</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="n">
+      <c r="A61" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="13" t="inlineStr">
+      <c r="B61" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:27</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>Add full social meta, PWA manifest, and app/Farcaster embeds</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="n">
+      <c r="A62" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="13" t="inlineStr">
+      <c r="B62" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:00</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>i18n: re-translate zh UI (replace machine-slop) + complete es gaps</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="n">
+      <c r="A63" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B63" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:07</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D63" s="15" t="inlineStr">
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>i18n: add French (fr) locale</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="n">
+      <c r="A64" s="10" t="n">
         <v>61</v>
       </c>
-      <c r="B64" s="13" t="inlineStr">
+      <c r="B64" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:18</t>
         </is>
       </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>Fix build: stop hardcoding /srv/www as vite outDir</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="n">
+      <c r="A65" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="B65" s="13" t="inlineStr">
+      <c r="B65" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:21</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D65" s="15" t="inlineStr">
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>i18n: accept fr in server locale enums (register, set-locale, admin, questions)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="n">
+      <c r="A66" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="B66" s="13" t="inlineStr">
+      <c r="B66" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:38</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D66" s="15" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
         <is>
           <t>docs: thorough Privacy Policy + Terms of Use (token/no-returns, liability)</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="n">
+      <c r="A67" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="B67" s="13" t="inlineStr">
+      <c r="B67" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 09:23</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D67" s="15" t="inlineStr">
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>docs: make web3 forward-looking for no-web3 launch; stash full token terms</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="n">
+      <c r="A68" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="13" t="inlineStr">
+      <c r="B68" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 09:57</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D68" s="15" t="inlineStr">
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
         <is>
           <t>ci: skip bushleague/labs demo deploy when DEPLOY_SSH_KEY is unset</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="n">
+      <c r="A69" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="B69" s="13" t="inlineStr">
+      <c r="B69" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 10:32</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>docs: add pre-launch review (findings for lead dev / legal / ops)</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="n">
+      <c r="A70" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="B70" s="13" t="inlineStr">
+      <c r="B70" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 11:49</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D70" s="15" t="inlineStr">
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
         <is>
           <t>fix(server): await migration async gaps in register + trivia/rush-hour answer paths</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="n">
+      <c r="A71" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="B71" s="13" t="inlineStr">
+      <c r="B71" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:08</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D71" s="15" t="inlineStr">
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
         <is>
           <t>[WIP] async-correctness sweep (NOT deployable yet — server tree does not compile clean)</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="13" t="n">
+      <c r="A72" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="B72" s="13" t="inlineStr">
+      <c r="B72" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:53</t>
         </is>
       </c>
-      <c r="C72" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>Fix MariaDB-migration async/await gaps across the server (full sweep)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="n">
+      <c r="A73" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="B73" s="13" t="inlineStr">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:57</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D73" s="15" t="inlineStr">
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>ci: exclude legacy server/src from server typecheck gate</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="n">
+      <c r="A74" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="B74" s="13" t="inlineStr">
+      <c r="B74" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 14:03</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>docs(roadmap): add staking to the deferred token terms (yield + partner undecided)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="n">
+      <c r="A75" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="B75" s="13" t="inlineStr">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 14:37</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>ui: fix guest CTA card spacing, surface docs on desktop, add placeholder CA pill</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="13" t="n">
+      <c r="A76" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="13" t="inlineStr">
+      <c r="B76" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 15:17</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
         <is>
           <t>fix: don't blank the app when /api/games returns a non-array</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="n">
+      <c r="A77" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="B77" s="13" t="inlineStr">
+      <c r="B77" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 16:43</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
         <is>
           <t>docs: add Roadmap page + purge bushleague from user-facing copy</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="13" t="n">
+      <c r="A78" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="B78" s="13" t="inlineStr">
+      <c r="B78" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 16:57</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
         <is>
           <t>chore: purge bushleague from everything in code (relic — it's only a host name)</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="13" t="n">
+      <c r="A79" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="B79" s="13" t="inlineStr">
+      <c r="B79" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:02</t>
         </is>
       </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
         <is>
           <t>chore: set official token contract address (CA pill)</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="n">
+      <c r="A80" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="13" t="inlineStr">
+      <c r="B80" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:16</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
         <is>
           <t>docs: reconcile chain references to Solana (token moved from BSC)</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="13" t="n">
+      <c r="A81" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="B81" s="13" t="inlineStr">
+      <c r="B81" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:56</t>
         </is>
       </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D81" s="12" t="inlineStr">
         <is>
           <t>docs: full Roadmap (vision, Now / 30-day / 60-day / Beyond)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="n">
+      <c r="A82" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="13" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:04</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D82" s="12" t="inlineStr">
         <is>
           <t>fix: trivia sounds = beeps/boops only + tighten quiz spacing</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="n">
+      <c r="A83" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="B83" s="13" t="inlineStr">
+      <c r="B83" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:41</t>
         </is>
       </c>
-      <c r="C83" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
         <is>
           <t>feat(web3): Solana holder-perks layer (web3.ruby-trivia.com)</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="13" t="n">
+      <c r="A84" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="13" t="inlineStr">
+      <c r="B84" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:49</t>
         </is>
       </c>
-      <c r="C84" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
         <is>
           <t>docs: prod backend handoff — master&lt;-&gt;MariaDB divergence (for Odi)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="13" t="n">
+      <c r="A85" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="B85" s="13" t="inlineStr">
+      <c r="B85" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 20:59</t>
         </is>
       </c>
-      <c r="C85" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D85" s="15" t="inlineStr">
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
         <is>
           <t>feat(web3 UI): wallet connect in bottom nav + polish (for Odi to integrate)</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="13" t="n">
+      <c r="A86" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="B86" s="13" t="inlineStr">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 22:50</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
         <is>
           <t>fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desktop wallet</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="13" t="n">
+      <c r="A87" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="B87" s="13" t="inlineStr">
+      <c r="B87" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:17</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D87" s="15" t="inlineStr">
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
         <is>
           <t>fix(web3): show wallet Connect in guest mode (sidebar + bottom nav)</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="13" t="n">
+      <c r="A88" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="13" t="inlineStr">
+      <c r="B88" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:24</t>
         </is>
       </c>
-      <c r="C88" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D88" s="15" t="inlineStr">
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
         <is>
           <t>fix(nav): guest desktop sidebar 1:1 with mobile bottom nav</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="13" t="n">
+      <c r="A89" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="B89" s="13" t="inlineStr">
+      <c r="B89" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:26</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D89" s="15" t="inlineStr">
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
         <is>
           <t>fix(i18n): add missing quiz.todaysQuiz key (was rendering raw "quiz.todaysQuiz")</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="13" t="n">
+      <c r="A90" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="B90" s="13" t="inlineStr">
+      <c r="B90" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:32</t>
         </is>
       </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D90" s="15" t="inlineStr">
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>i18n(web3): translate wallet-modal strings into all locales</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="13" t="n">
+      <c r="A91" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="B91" s="13" t="inlineStr">
+      <c r="B91" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:40</t>
         </is>
       </c>
-      <c r="C91" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D91" s="15" t="inlineStr">
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
         <is>
           <t>fix(i18n): translate practice-topic category labels</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="13" t="n">
+      <c r="A92" s="10" t="n">
         <v>89</v>
       </c>
-      <c r="B92" s="13" t="inlineStr">
+      <c r="B92" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:48</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D92" s="15" t="inlineStr">
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
         <is>
           <t>fix(guest): restore Sign in / Create account CTA on guest profile (mobile login)</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="13" t="n">
+      <c r="A93" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="B93" s="13" t="inlineStr">
+      <c r="B93" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 00:08</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D93" s="15" t="inlineStr">
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
         <is>
           <t>fix(deploy): kill labs subdomain — labs.ruby-trivia.com → www.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="13" t="n">
+      <c r="A94" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="B94" s="13" t="inlineStr">
+      <c r="B94" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 00:28</t>
         </is>
       </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D94" s="15" t="inlineStr">
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
         <is>
           <t>fix(deploy): actually build + ship the web3 bundle to web3.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="13" t="n">
+      <c r="A95" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="B95" s="13" t="inlineStr">
+      <c r="B95" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 01:10</t>
         </is>
       </c>
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D95" s="15" t="inlineStr">
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
         <is>
           <t>fix(web3): error-boundary the wallet nav button so it can't take down the nav</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="13" t="n">
+      <c r="A96" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="13" t="inlineStr">
+      <c r="B96" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 02:21</t>
         </is>
       </c>
-      <c r="C96" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D96" s="15" t="inlineStr">
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
         <is>
           <t>docs: fix stale BNB Smart Chain refs (token is live on Solana)</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="13" t="n">
+      <c r="A97" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="B97" s="13" t="inlineStr">
+      <c r="B97" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 02:26</t>
         </is>
       </c>
-      <c r="C97" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D97" s="15" t="inlineStr">
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
         <is>
           <t>docs: token ticker is $TRIVIA, not RUBY (Ruby Trivia is the game)</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="13" t="n">
+      <c r="A98" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="13" t="inlineStr">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 04:50</t>
         </is>
       </c>
-      <c r="C98" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D98" s="15" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D98" s="12" t="inlineStr">
         <is>
           <t>feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="13" t="n">
+      <c r="A99" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="B99" s="13" t="inlineStr">
+      <c r="B99" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C99" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D99" s="15" t="inlineStr">
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="13" t="n">
+      <c r="A100" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="13" t="inlineStr">
+      <c r="B100" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D100" s="15" t="inlineStr">
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D100" s="12" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="13" t="n">
+      <c r="A101" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="B101" s="13" t="inlineStr">
+      <c r="B101" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 15:49</t>
         </is>
       </c>
-      <c r="C101" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D101" s="15" t="inlineStr">
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr">
         <is>
           <t>fix(web2): hide token CA pill in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="13" t="n">
+      <c r="A102" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="13" t="inlineStr">
+      <c r="B102" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 15:53</t>
         </is>
       </c>
-      <c r="C102" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D102" s="15" t="inlineStr">
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
         <is>
           <t>fix(web2): hide tokenomics docs article in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="13" t="n">
+      <c r="A103" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="B103" s="13" t="inlineStr">
+      <c r="B103" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 16:39</t>
         </is>
       </c>
-      <c r="C103" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D103" s="15" t="inlineStr">
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
         <is>
           <t>feat(store): ship native app as free v1 (no subscribe stub)</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="13" t="n">
+      <c r="A104" s="10" t="n">
         <v>101</v>
       </c>
-      <c r="B104" s="13" t="inlineStr">
+      <c r="B104" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 16:47</t>
         </is>
       </c>
-      <c r="C104" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D104" s="15" t="inlineStr">
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
         <is>
           <t>feat(live): resilient WS reconnect — backoff, auto-rejoin, graceful fail</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="13" t="n">
+      <c r="A105" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="B105" s="13" t="inlineStr">
+      <c r="B105" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 17:44</t>
         </is>
       </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D105" s="15" t="inlineStr">
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="inlineStr">
         <is>
           <t>docs: app-store distribution plan + session handoff</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="13" t="n">
+      <c r="A106" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="B106" s="13" t="inlineStr">
+      <c r="B106" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 18:12</t>
         </is>
       </c>
-      <c r="C106" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D106" s="15" t="inlineStr">
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D106" s="12" t="inlineStr">
         <is>
           <t>feat(live): broadcast stage view of live trivia rounds (P0)</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="13" t="n">
+      <c r="A107" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="B107" s="13" t="inlineStr">
+      <c r="B107" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 18:22</t>
         </is>
       </c>
-      <c r="C107" s="13" t="inlineStr">
+      <c r="C107" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D107" s="15" t="inlineStr">
+      <c r="D107" s="12" t="inlineStr">
         <is>
           <t>Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcbd610a5	2026-06-26T13:45:01-04:00	ruby-trivia-handbook	Handbook: add public titles (Dutch = lead dev, Odi = lead marketing); both doing both</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="13" t="n">
+      <c r="A108" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="B108" s="13" t="inlineStr">
+      <c r="B108" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 09:37</t>
         </is>
       </c>
-      <c r="C108" s="13" t="inlineStr">
+      <c r="C108" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D108" s="15" t="inlineStr">
+      <c r="D108" s="12" t="inlineStr">
         <is>
           <t>Add manager planning set: state-of-project, idea bank, roadmap, 1/3/7/14/30-day deliverables, team instructions, risks/ops</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="13" t="n">
+      <c r="A109" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="B109" s="13" t="inlineStr">
+      <c r="B109" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:00</t>
         </is>
       </c>
-      <c r="C109" s="13" t="inlineStr">
+      <c r="C109" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D109" s="15" t="inlineStr">
+      <c r="D109" s="12" t="inlineStr">
         <is>
           <t>Sensitivity pass: soften ownership language, ease comp/financials, pull Chess in, detail Day 3</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="13" t="n">
+      <c r="A110" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="B110" s="13" t="inlineStr">
+      <c r="B110" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:13</t>
         </is>
       </c>
-      <c r="C110" s="13" t="inlineStr">
+      <c r="C110" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D110" s="15" t="inlineStr">
+      <c r="D110" s="12" t="inlineStr">
         <is>
           <t>Correct for Magic's departure + add weekend primer</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="13" t="n">
+      <c r="A111" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="B111" s="13" t="inlineStr">
+      <c r="B111" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:24</t>
         </is>
       </c>
-      <c r="C111" s="13" t="inlineStr">
+      <c r="C111" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D111" s="15" t="inlineStr">
+      <c r="D111" s="12" t="inlineStr">
         <is>
           <t>Weekend primer: Lotus/itachi = consultants, Odi runs X, + Saturday Space, challenge-to-play, example posts</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="13" t="n">
+      <c r="A112" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="B112" s="13" t="inlineStr">
+      <c r="B112" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:35</t>
         </is>
       </c>
-      <c r="C112" s="13" t="inlineStr">
+      <c r="C112" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D112" s="15" t="inlineStr">
+      <c r="D112" s="12" t="inlineStr">
         <is>
           <t>Scrub all 'bundle' mentions; reframe Bao/nerd + Lotus/itachi as outside (not team)</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="13" t="n">
+      <c r="A113" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="B113" s="13" t="inlineStr">
+      <c r="B113" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:47</t>
         </is>
       </c>
-      <c r="C113" s="13" t="inlineStr">
+      <c r="C113" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D113" s="15" t="inlineStr">
+      <c r="D113" s="12" t="inlineStr">
         <is>
           <t>Add X Space talking-points cheat sheet (Sat) — beats, soundbites, hard-Q answers, guardrails</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="13" t="n">
+      <c r="A114" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="B114" s="13" t="inlineStr">
+      <c r="B114" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:51</t>
         </is>
       </c>
-      <c r="C114" s="13" t="inlineStr">
+      <c r="C114" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D114" s="15" t="inlineStr">
+      <c r="D114" s="12" t="inlineStr">
         <is>
           <t>Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6bf157372e19db43bc75fda	2026-06-26T15:58:55-04:00	ruby-trivia	docs(web3): independent legal/regulatory research report</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="13" t="n">
+      <c r="A115" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="B115" s="13" t="inlineStr">
+      <c r="B115" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:59</t>
         </is>
       </c>
-      <c r="C115" s="13" t="inlineStr">
+      <c r="C115" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
+      <c r="D115" s="12" t="inlineStr">
         <is>
           <t>Strip theme banner; landing page = just the team + weekend links (nothing above)</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="13" t="n">
+      <c r="A116" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="B116" s="13" t="inlineStr">
+      <c r="B116" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:04</t>
         </is>
       </c>
-      <c r="C116" s="13" t="inlineStr">
+      <c r="C116" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
+      <c r="D116" s="12" t="inlineStr">
         <is>
           <t>Weekend page: put the actionable plan back (X post examples, thread, challenge copy, Space) — minus internal-only bits</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="13" t="n">
+      <c r="A117" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="B117" s="13" t="inlineStr">
+      <c r="B117" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:09</t>
         </is>
       </c>
-      <c r="C117" s="13" t="inlineStr">
+      <c r="C117" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D117" s="15" t="inlineStr">
+      <c r="D117" s="12" t="inlineStr">
         <is>
           <t>Add public FAQ (hard questions, cleaned) + link from landing</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="13" t="n">
+      <c r="A118" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="B118" s="13" t="inlineStr">
+      <c r="B118" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:16</t>
         </is>
       </c>
-      <c r="C118" s="13" t="inlineStr">
+      <c r="C118" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D118" s="15" t="inlineStr">
+      <c r="D118" s="12" t="inlineStr">
         <is>
           <t>Team: Dutch + Odi are the two-person core, tied across everything (not split by frontend/backend)</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="13" t="n">
+      <c r="A119" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="B119" s="13" t="inlineStr">
+      <c r="B119" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:23</t>
         </is>
       </c>
-      <c r="C119" s="13" t="inlineStr">
+      <c r="C119" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D119" s="15" t="inlineStr">
+      <c r="D119" s="12" t="inlineStr">
         <is>
           <t>Clarify: posts are examples to work from (not post-as-is); designate X = Odi; community = TG (Destiny), not X</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="13" t="n">
+      <c r="A120" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="B120" s="13" t="inlineStr">
+      <c r="B120" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:39</t>
         </is>
       </c>
-      <c r="C120" s="13" t="inlineStr">
+      <c r="C120" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D120" s="15" t="inlineStr">
+      <c r="D120" s="12" t="inlineStr">
         <is>
           <t>Sync private docs to handbook: Dutch+Odi tied across everything; toolkit = examples to work from (not canned posts)</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="13" t="n">
+      <c r="A121" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="B121" s="13" t="inlineStr">
+      <c r="B121" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 12:51</t>
         </is>
       </c>
-      <c r="C121" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D121" s="15" t="inlineStr">
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="inlineStr">
         <is>
           <t>feat(bot): /stats — lifetime avg points per question &amp; per round</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="13" t="n">
+      <c r="A122" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="B122" s="13" t="inlineStr">
+      <c r="B122" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 13:44</t>
         </is>
       </c>
-      <c r="C122" s="13" t="inlineStr">
+      <c r="C122" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D122" s="15" t="inlineStr">
+      <c r="D122" s="12" t="inlineStr">
         <is>
           <t>Titles + decision structure + capacity/slow-roll across planning set</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="13" t="n">
+      <c r="A123" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="B123" s="13" t="inlineStr">
+      <c r="B123" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 13:45</t>
         </is>
       </c>
-      <c r="C123" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D123" s="15" t="inlineStr">
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="inlineStr">
         <is>
           <t>feat(stats): efficiency averages across all telegram modes + web profile</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="13" t="n">
+      <c r="A124" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="B124" s="13" t="inlineStr">
+      <c r="B124" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 15:53</t>
         </is>
       </c>
-      <c r="C124" s="13" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D124" s="15" t="inlineStr">
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
         <is>
           <t>docs(web3): branch for tokenomics/NFT work + compliance guardrails</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="13" t="n">
+      <c r="A125" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="B125" s="13" t="inlineStr">
+      <c r="B125" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:04</t>
         </is>
       </c>
-      <c r="C125" s="13" t="inlineStr">
+      <c r="C125" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D125" s="15" t="inlineStr">
+      <c r="D125" s="12" t="inlineStr">
         <is>
           <t>Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel web2/web3, risk-parity control)</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="13" t="n">
+      <c r="A126" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="B126" s="13" t="inlineStr">
+      <c r="B126" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:10</t>
         </is>
       </c>
-      <c r="C126" s="13" t="inlineStr">
+      <c r="C126" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D126" s="15" t="inlineStr">
+      <c r="D126" s="12" t="inlineStr">
         <is>
           <t>Add 07: tax &amp; legal/regulatory research (cited) for the governance structure</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="13" t="n">
+      <c r="A127" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="B127" s="13" t="inlineStr">
+      <c r="B127" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:17</t>
         </is>
       </c>
-      <c r="C127" s="13" t="inlineStr">
+      <c r="C127" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D127" s="15" t="inlineStr">
+      <c r="D127" s="12" t="inlineStr">
         <is>
           <t>Add 08: latest 2025-26 statutes + how-others-do-it playbooks + right-sized recommended path</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="13" t="n">
+      <c r="A128" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="B128" s="13" t="inlineStr">
+      <c r="B128" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:05</t>
         </is>
       </c>
-      <c r="C128" s="13" t="inlineStr">
+      <c r="C128" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D128" s="15" t="inlineStr">
+      <c r="D128" s="12" t="inlineStr">
         <is>
           <t>Add browsable docs hub (README front page) + S-corp analysis across 06/07/08</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="13" t="n">
+      <c r="A129" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="B129" s="13" t="inlineStr">
+      <c r="B129" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:22</t>
         </is>
       </c>
-      <c r="C129" s="13" t="inlineStr">
+      <c r="C129" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D129" s="15" t="inlineStr">
+      <c r="D129" s="12" t="inlineStr">
         <is>
           <t>Add founder/operator compensation working proposal (24h counter window) to 06; thread through 07/08/README</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="13" t="n">
+      <c r="A130" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="B130" s="13" t="inlineStr">
+      <c r="B130" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:50</t>
         </is>
       </c>
-      <c r="C130" s="13" t="inlineStr">
+      <c r="C130" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D130" s="15" t="inlineStr">
+      <c r="D130" s="12" t="inlineStr">
         <is>
           <t>Comp: operator draw is CAPPED at a fair daily wage (excess stays in treasury)</t>
         </is>
@@ -3930,28 +3865,28 @@
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>• Hours from GitHub commit timestamps. Floor = git-hours method (&gt;2h gap=new session, +2h ramp). Realistic = active-day method weighted by commit intensity (heaviest day ~16h, normal active day ~8h).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>• All commits under 'dutch &lt;dutchiono@gmail.com&gt;' / GitHub 'dutchiono' across all Ruby repos. Other contributors excluded.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>• Date range 2026-05-29 to 2026-06-29; 13 active days; 127 commits.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>• Amount paid to date: $350. Three rate scenarios: $10, $50, $150/hr.</t>
         </is>

</xml_diff>

<commit_message>
Reframe as Bill + Bid: vertical invoice (amount due $4,950 @ agreed $50), clean tables, real download
</commit_message>
<xml_diff>
--- a/Dutch-Ruby-Comp-Claim.xlsx
+++ b/Dutch-Ruby-Comp-Claim.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bid" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bill &amp; Bid" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hours by Day" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What was built" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commit Log" sheetId="4" state="visible" r:id="rId4"/>
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -89,14 +93,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -486,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -499,7 +505,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ruby Trivia — Hours &amp; Bid (Dutch / dutchiono)</t>
+          <t>Ruby Trivia — Bill &amp; Bid (Dutch / dutchiono)</t>
         </is>
       </c>
     </row>
@@ -563,84 +569,101 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>AMOUNT DUE  (106 hrs × $50 agreed − $350 paid)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>4950</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BID — the same hours at three rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Owed</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>$10/hr</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>106</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C15" s="10" t="n">
         <v>1060</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D15" s="10" t="n">
         <v>350</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E15" s="11" t="n">
         <v>710</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>$25/hr</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B16" s="9" t="n">
         <v>106</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C16" s="10" t="n">
         <v>2650</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D16" s="10" t="n">
         <v>350</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E16" s="11" t="n">
         <v>2300</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>$50/hr</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B17" s="9" t="n">
         <v>106</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C17" s="10" t="n">
         <v>5300</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D17" s="10" t="n">
         <v>350</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E17" s="11" t="n">
         <v>4950</v>
       </c>
     </row>
@@ -676,458 +699,458 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Commits</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Hrs</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>@ $10</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>@ $25</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>@ $50</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Repos / sample work</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ru</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">ruby-trivia — untracked files on iono/games-production: dc3e01f Archive iono games production </t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>ruby-labs — Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="13" t="n">
         <v>160</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — CI: use plain bun install (lockfile drifts across bun versions) + resync bun.loc</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="13" t="n">
         <v>160</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>ruby-trivia — fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia — Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcb</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia, ruby-trivia-handbook — Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>ruby-marketing — Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel we</t>
         </is>
@@ -1146,13 +1169,13 @@
       <c r="D17" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="15" t="n">
         <v>1060</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="15" t="n">
         <v>2650</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="15" t="n">
         <v>5300</v>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1182,70 +1205,70 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>• Trivia PWA — daily quiz, practice, friend challenges, leaderboards, streaks, ranks/badges, 4 languages, installable</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>• Live multiplayer — realtime WebSocket lobbies, matchmaking, graceful reconnect</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>• Backend &amp; API — Hono/Bun server, auth/registration, game logic, SQLite→MariaDB migration + SQL translation</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>• Web3 holder layer — Solana wallet connect, holder verification, perks (multiplier, holders-only leaderboard, cosmetics)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>• On-chain / contracts — contract suite, result-signer seam, token integration</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>• Telegram bot gateway — in-chat trivia, stateless solo play, /stats</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>• Production infra / DevOps — multi-container, nginx, MariaDB, deploy scripts, live incident response</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>• App-store repackaging — Capacitor + multi-store editions</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>• Token launch support &amp; ops — Solana/Pump.fun launch, splash/CA, coordination</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>• Educational variant — ruby-trivia-classroom</t>
         </is>
@@ -1279,2562 +1302,2562 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Date / time</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Repo</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>2026-05-29 22:58</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ruby-labs	feat: sync latest marketing landing from ruby-trivia + i18n; purge bushleague</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 10:58</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Ship Ruby Trivia classroom hub with library-themed UI for bushleague.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:41</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Fix shelf book launches, clay UI, classroom sounds and haptics.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Mobile-first layout and full main-repo trivia parity.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Fix deploy script staging cleanup on Windows.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:47</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:49</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Fix GitHub Actions deploy SSH key and scp paths.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:51</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Fix CI deploy rsync when scp nests files under dist/.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 22:56</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Remove Class from header; rename nav to Lessons.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:00</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Boost clay depth and sounds; drop fake leaderboard names.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:03</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Replace open Create with curated quiz sets; drop unsigned custom questions.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:04</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Fix nav sounds: play on tab click inside user gesture.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:05</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Stop defaulting player name to Ruby; clear persisted Ruby names.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:07</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Block Ruby as player name; no anonymous leaderboard rows.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:08</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Add preferred Ruby Trivia logo to header.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:10</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Omit unnamed players from scoreboards; document backend contract.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:12</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Put Trivia above Lessons in nav.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>2026-06-16 23:14</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Remove duplicate hero logo; use downloaded sound files for cues.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>2026-06-17 22:12</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>2026-06-17 22:15</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Fix deploy script line endings and static upload cleanup.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>2026-06-18 17:15</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>2026-06-18 17:28</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Restructure mobile nav around Games hub and add Odie's Car.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>2026-06-18 22:45</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Add Bush League clay dress kit and apply theme to app shell.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="n">
+      <c r="A27" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>2026-06-19 14:33</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n">
+      <c r="A28" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>2026-06-19 14:34</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Add single-repo workflow doc after consolidating on ruby-high/ruby-trivia.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="n">
+      <c r="A29" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>index on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>untracked files on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="n">
+      <c r="A31" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e675af6ce46b	2026-06-25T04:50:33-04:00	dutchiono-ruby-trivia	feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n">
+      <c r="A32" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Ignore TypeScript build info files.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="n">
+      <c r="A33" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>2026-06-21 02:51</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n">
+      <c r="A34" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 13:23</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="n">
+      <c r="A35" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 13:27</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>Add auth intent persistence and fix live room invite flow.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n">
+      <c r="A36" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 13:33</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>Harden anotherone deploy: exclude server node_modules from upload.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="n">
+      <c r="A37" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 13:37</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>Fix unreadable theme-option buttons on clay cards in dark mode.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="n">
+      <c r="A38" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 14:45</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>Add side dock rail, RUBYSQUARE header mark, and clay contrast fixes.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="n">
+      <c r="A39" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>2026-06-22 21:22</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>Remove third-party studio branding and add session handoff doc.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n">
+      <c r="A40" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 06:22</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>Document single-branch workflow; rename archive branch.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="n">
+      <c r="A41" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="n">
+      <c r="A42" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="10" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="n">
+      <c r="A43" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="n">
+      <c r="A44" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="n">
+      <c r="A45" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 11:22</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Use MP3-only sensory assets from Audacity exports.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="n">
+      <c r="A46" s="12" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 11:29</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D46" s="12" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>Add on-chain scaffold, chain signer API, brand assets, and trivia data.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="n">
+      <c r="A47" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="10" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 11:40</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>Show Ruby Trivia logo in minimized mobile header chrome.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="n">
+      <c r="A48" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 12:09</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>Fix minimized mobile header: slim RUBYSQUARE pill, no side rail.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="n">
+      <c r="A49" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 12:29</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
         <is>
           <t>Route nav sounds: zipper on top dock, page on bottom subnav, paper on ranks.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="n">
+      <c r="A50" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 15:56</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D50" s="12" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>Refactor trivia navigation: bottom nav, mode nav, games layout</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="n">
+      <c r="A51" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="10" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 18:26</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D51" s="12" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>Fix unreadable secondary buttons on cream modals</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="n">
+      <c r="A52" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 19:46</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D52" s="12" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
         <is>
           <t>Fix missing desktop nav rail in authenticated layout</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="n">
+      <c r="A53" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:02</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D53" s="12" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
         <is>
           <t>Warm blue chrome to clay palette + add Docs to desktop nav</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="n">
+      <c r="A54" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:07</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>Reskin splash CTA from blue to clay orange</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="n">
+      <c r="A55" s="12" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:09</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D55" s="12" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>Warm active language-picker chip to clay orange</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="n">
+      <c r="A56" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="10" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:12</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D56" s="12" t="inlineStr">
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>Warm language-button focus outline to clay orange</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="10" t="n">
+      <c r="A57" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B57" s="10" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:34</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D57" s="12" t="inlineStr">
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>Public /docs route, clay answer buttons, warm crew links</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="10" t="n">
+      <c r="A58" s="12" t="n">
         <v>55</v>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 20:43</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D58" s="12" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>Fix production DB corruption: stop deploy from clobbering the live SQLite db</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="10" t="n">
+      <c r="A59" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B59" s="10" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 21:06</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>Add PR CI: build + chain tests</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="n">
+      <c r="A60" s="12" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 21:08</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>CI: use plain bun install (lockfile drifts across bun versions) + resync bun.lock</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="n">
+      <c r="A61" s="12" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>2026-06-23 21:27</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>Add full social meta, PWA manifest, and app/Farcaster embeds</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="n">
+      <c r="A62" s="12" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="10" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 08:00</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D62" s="12" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>i18n: re-translate zh UI (replace machine-slop) + complete es gaps</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="n">
+      <c r="A63" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B63" s="10" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 08:07</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D63" s="12" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>i18n: add French (fr) locale</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="10" t="n">
+      <c r="A64" s="12" t="n">
         <v>61</v>
       </c>
-      <c r="B64" s="10" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 08:18</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>Fix build: stop hardcoding /srv/www as vite outDir</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="n">
+      <c r="A65" s="12" t="n">
         <v>62</v>
       </c>
-      <c r="B65" s="10" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 08:21</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D65" s="12" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>i18n: accept fr in server locale enums (register, set-locale, admin, questions)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="n">
+      <c r="A66" s="12" t="n">
         <v>63</v>
       </c>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 08:38</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D66" s="12" t="inlineStr">
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>docs: thorough Privacy Policy + Terms of Use (token/no-returns, liability)</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="n">
+      <c r="A67" s="12" t="n">
         <v>64</v>
       </c>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 09:23</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D67" s="12" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
         <is>
           <t>docs: make web3 forward-looking for no-web3 launch; stash full token terms</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="n">
+      <c r="A68" s="12" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="10" t="inlineStr">
+      <c r="B68" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 09:57</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>ci: skip bushleague/labs demo deploy when DEPLOY_SSH_KEY is unset</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="n">
+      <c r="A69" s="12" t="n">
         <v>66</v>
       </c>
-      <c r="B69" s="10" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 10:32</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D69" s="12" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>docs: add pre-launch review (findings for lead dev / legal / ops)</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="n">
+      <c r="A70" s="12" t="n">
         <v>67</v>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 11:49</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D70" s="12" t="inlineStr">
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>fix(server): await migration async gaps in register + trivia/rush-hour answer paths</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="n">
+      <c r="A71" s="12" t="n">
         <v>68</v>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 12:08</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D71" s="12" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
         <is>
           <t>[WIP] async-correctness sweep (NOT deployable yet — server tree does not compile clean)</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="n">
+      <c r="A72" s="12" t="n">
         <v>69</v>
       </c>
-      <c r="B72" s="10" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 12:53</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D72" s="12" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
         <is>
           <t>Fix MariaDB-migration async/await gaps across the server (full sweep)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="10" t="n">
+      <c r="A73" s="12" t="n">
         <v>70</v>
       </c>
-      <c r="B73" s="10" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 12:57</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D73" s="12" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
         <is>
           <t>ci: exclude legacy server/src from server typecheck gate</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="10" t="n">
+      <c r="A74" s="12" t="n">
         <v>71</v>
       </c>
-      <c r="B74" s="10" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 14:03</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D74" s="12" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
         <is>
           <t>docs(roadmap): add staking to the deferred token terms (yield + partner undecided)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="10" t="n">
+      <c r="A75" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="B75" s="10" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 14:37</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D75" s="12" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
         <is>
           <t>ui: fix guest CTA card spacing, surface docs on desktop, add placeholder CA pill</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="10" t="n">
+      <c r="A76" s="12" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="10" t="inlineStr">
+      <c r="B76" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 15:17</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D76" s="12" t="inlineStr">
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
         <is>
           <t>fix: don't blank the app when /api/games returns a non-array</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="n">
+      <c r="A77" s="12" t="n">
         <v>74</v>
       </c>
-      <c r="B77" s="10" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 16:43</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D77" s="12" t="inlineStr">
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
         <is>
           <t>docs: add Roadmap page + purge bushleague from user-facing copy</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="10" t="n">
+      <c r="A78" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="B78" s="10" t="inlineStr">
+      <c r="B78" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 16:57</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D78" s="12" t="inlineStr">
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
         <is>
           <t>chore: purge bushleague from everything in code (relic — it's only a host name)</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="n">
+      <c r="A79" s="12" t="n">
         <v>76</v>
       </c>
-      <c r="B79" s="10" t="inlineStr">
+      <c r="B79" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 17:02</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D79" s="12" t="inlineStr">
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
         <is>
           <t>chore: set official token contract address (CA pill)</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="10" t="n">
+      <c r="A80" s="12" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="10" t="inlineStr">
+      <c r="B80" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 17:16</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D80" s="12" t="inlineStr">
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
         <is>
           <t>docs: reconcile chain references to Solana (token moved from BSC)</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="10" t="n">
+      <c r="A81" s="12" t="n">
         <v>78</v>
       </c>
-      <c r="B81" s="10" t="inlineStr">
+      <c r="B81" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 17:56</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D81" s="12" t="inlineStr">
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
         <is>
           <t>docs: full Roadmap (vision, Now / 30-day / 60-day / Beyond)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="n">
+      <c r="A82" s="12" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="10" t="inlineStr">
+      <c r="B82" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 19:04</t>
         </is>
       </c>
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D82" s="12" t="inlineStr">
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
         <is>
           <t>fix: trivia sounds = beeps/boops only + tighten quiz spacing</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="n">
+      <c r="A83" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="B83" s="10" t="inlineStr">
+      <c r="B83" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 19:41</t>
         </is>
       </c>
-      <c r="C83" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D83" s="12" t="inlineStr">
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
         <is>
           <t>feat(web3): Solana holder-perks layer (web3.ruby-trivia.com)</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="10" t="n">
+      <c r="A84" s="12" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="10" t="inlineStr">
+      <c r="B84" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 19:49</t>
         </is>
       </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D84" s="12" t="inlineStr">
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
         <is>
           <t>docs: prod backend handoff — master&lt;-&gt;MariaDB divergence (for Odi)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="10" t="n">
+      <c r="A85" s="12" t="n">
         <v>82</v>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B85" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 20:59</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D85" s="12" t="inlineStr">
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
         <is>
           <t>feat(web3 UI): wallet connect in bottom nav + polish (for Odi to integrate)</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="n">
+      <c r="A86" s="12" t="n">
         <v>83</v>
       </c>
-      <c r="B86" s="10" t="inlineStr">
+      <c r="B86" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 22:50</t>
         </is>
       </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D86" s="12" t="inlineStr">
+      <c r="C86" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
         <is>
           <t>fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desktop wallet</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="10" t="n">
+      <c r="A87" s="12" t="n">
         <v>84</v>
       </c>
-      <c r="B87" s="10" t="inlineStr">
+      <c r="B87" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:17</t>
         </is>
       </c>
-      <c r="C87" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D87" s="12" t="inlineStr">
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
         <is>
           <t>fix(web3): show wallet Connect in guest mode (sidebar + bottom nav)</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="10" t="n">
+      <c r="A88" s="12" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="10" t="inlineStr">
+      <c r="B88" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:24</t>
         </is>
       </c>
-      <c r="C88" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D88" s="12" t="inlineStr">
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
         <is>
           <t>fix(nav): guest desktop sidebar 1:1 with mobile bottom nav</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="10" t="n">
+      <c r="A89" s="12" t="n">
         <v>86</v>
       </c>
-      <c r="B89" s="10" t="inlineStr">
+      <c r="B89" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:26</t>
         </is>
       </c>
-      <c r="C89" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D89" s="12" t="inlineStr">
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
         <is>
           <t>fix(i18n): add missing quiz.todaysQuiz key (was rendering raw "quiz.todaysQuiz")</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="10" t="n">
+      <c r="A90" s="12" t="n">
         <v>87</v>
       </c>
-      <c r="B90" s="10" t="inlineStr">
+      <c r="B90" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:32</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D90" s="12" t="inlineStr">
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
         <is>
           <t>i18n(web3): translate wallet-modal strings into all locales</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="10" t="n">
+      <c r="A91" s="12" t="n">
         <v>88</v>
       </c>
-      <c r="B91" s="10" t="inlineStr">
+      <c r="B91" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:40</t>
         </is>
       </c>
-      <c r="C91" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D91" s="12" t="inlineStr">
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
         <is>
           <t>fix(i18n): translate practice-topic category labels</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="10" t="n">
+      <c r="A92" s="12" t="n">
         <v>89</v>
       </c>
-      <c r="B92" s="10" t="inlineStr">
+      <c r="B92" s="12" t="inlineStr">
         <is>
           <t>2026-06-24 23:48</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D92" s="12" t="inlineStr">
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
         <is>
           <t>fix(guest): restore Sign in / Create account CTA on guest profile (mobile login)</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="10" t="n">
+      <c r="A93" s="12" t="n">
         <v>90</v>
       </c>
-      <c r="B93" s="10" t="inlineStr">
+      <c r="B93" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 00:08</t>
         </is>
       </c>
-      <c r="C93" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D93" s="12" t="inlineStr">
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
         <is>
           <t>fix(deploy): kill labs subdomain — labs.ruby-trivia.com → www.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="10" t="n">
+      <c r="A94" s="12" t="n">
         <v>91</v>
       </c>
-      <c r="B94" s="10" t="inlineStr">
+      <c r="B94" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 00:28</t>
         </is>
       </c>
-      <c r="C94" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D94" s="12" t="inlineStr">
+      <c r="C94" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
         <is>
           <t>fix(deploy): actually build + ship the web3 bundle to web3.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="10" t="n">
+      <c r="A95" s="12" t="n">
         <v>92</v>
       </c>
-      <c r="B95" s="10" t="inlineStr">
+      <c r="B95" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 01:10</t>
         </is>
       </c>
-      <c r="C95" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D95" s="12" t="inlineStr">
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
         <is>
           <t>fix(web3): error-boundary the wallet nav button so it can't take down the nav</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="10" t="n">
+      <c r="A96" s="12" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="10" t="inlineStr">
+      <c r="B96" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 02:21</t>
         </is>
       </c>
-      <c r="C96" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D96" s="12" t="inlineStr">
+      <c r="C96" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
         <is>
           <t>docs: fix stale BNB Smart Chain refs (token is live on Solana)</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="10" t="n">
+      <c r="A97" s="12" t="n">
         <v>94</v>
       </c>
-      <c r="B97" s="10" t="inlineStr">
+      <c r="B97" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 02:26</t>
         </is>
       </c>
-      <c r="C97" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D97" s="12" t="inlineStr">
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
         <is>
           <t>docs: token ticker is $TRIVIA, not RUBY (Ruby Trivia is the game)</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="10" t="n">
+      <c r="A98" s="12" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="10" t="inlineStr">
+      <c r="B98" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 04:50</t>
         </is>
       </c>
-      <c r="C98" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D98" s="12" t="inlineStr">
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
         <is>
           <t>feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="10" t="n">
+      <c r="A99" s="12" t="n">
         <v>96</v>
       </c>
-      <c r="B99" s="10" t="inlineStr">
+      <c r="B99" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C99" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D99" s="12" t="inlineStr">
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="10" t="n">
+      <c r="A100" s="12" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="10" t="inlineStr">
+      <c r="B100" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C100" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D100" s="12" t="inlineStr">
+      <c r="C100" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="10" t="n">
+      <c r="A101" s="12" t="n">
         <v>98</v>
       </c>
-      <c r="B101" s="10" t="inlineStr">
+      <c r="B101" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 15:49</t>
         </is>
       </c>
-      <c r="C101" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D101" s="12" t="inlineStr">
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
         <is>
           <t>fix(web2): hide token CA pill in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="10" t="n">
+      <c r="A102" s="12" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="10" t="inlineStr">
+      <c r="B102" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 15:53</t>
         </is>
       </c>
-      <c r="C102" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D102" s="12" t="inlineStr">
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
         <is>
           <t>fix(web2): hide tokenomics docs article in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="n">
+      <c r="A103" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="B103" s="10" t="inlineStr">
+      <c r="B103" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 16:39</t>
         </is>
       </c>
-      <c r="C103" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D103" s="12" t="inlineStr">
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
         <is>
           <t>feat(store): ship native app as free v1 (no subscribe stub)</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="10" t="n">
+      <c r="A104" s="12" t="n">
         <v>101</v>
       </c>
-      <c r="B104" s="10" t="inlineStr">
+      <c r="B104" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 16:47</t>
         </is>
       </c>
-      <c r="C104" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D104" s="12" t="inlineStr">
+      <c r="C104" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>feat(live): resilient WS reconnect — backoff, auto-rejoin, graceful fail</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="10" t="n">
+      <c r="A105" s="12" t="n">
         <v>102</v>
       </c>
-      <c r="B105" s="10" t="inlineStr">
+      <c r="B105" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 17:44</t>
         </is>
       </c>
-      <c r="C105" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D105" s="12" t="inlineStr">
+      <c r="C105" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
         <is>
           <t>docs: app-store distribution plan + session handoff</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="n">
+      <c r="A106" s="12" t="n">
         <v>103</v>
       </c>
-      <c r="B106" s="10" t="inlineStr">
+      <c r="B106" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 18:12</t>
         </is>
       </c>
-      <c r="C106" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D106" s="12" t="inlineStr">
+      <c r="C106" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
         <is>
           <t>feat(live): broadcast stage view of live trivia rounds (P0)</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="n">
+      <c r="A107" s="12" t="n">
         <v>104</v>
       </c>
-      <c r="B107" s="10" t="inlineStr">
+      <c r="B107" s="12" t="inlineStr">
         <is>
           <t>2026-06-25 18:22</t>
         </is>
       </c>
-      <c r="C107" s="10" t="inlineStr">
+      <c r="C107" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D107" s="12" t="inlineStr">
+      <c r="D107" s="14" t="inlineStr">
         <is>
           <t>Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcbd610a5	2026-06-26T13:45:01-04:00	ruby-trivia-handbook	Handbook: add public titles (Dutch = lead dev, Odi = lead marketing); both doing both</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="10" t="n">
+      <c r="A108" s="12" t="n">
         <v>105</v>
       </c>
-      <c r="B108" s="10" t="inlineStr">
+      <c r="B108" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 09:37</t>
         </is>
       </c>
-      <c r="C108" s="10" t="inlineStr">
+      <c r="C108" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D108" s="12" t="inlineStr">
+      <c r="D108" s="14" t="inlineStr">
         <is>
           <t>Add manager planning set: state-of-project, idea bank, roadmap, 1/3/7/14/30-day deliverables, team instructions, risks/ops</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="10" t="n">
+      <c r="A109" s="12" t="n">
         <v>106</v>
       </c>
-      <c r="B109" s="10" t="inlineStr">
+      <c r="B109" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:00</t>
         </is>
       </c>
-      <c r="C109" s="10" t="inlineStr">
+      <c r="C109" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D109" s="12" t="inlineStr">
+      <c r="D109" s="14" t="inlineStr">
         <is>
           <t>Sensitivity pass: soften ownership language, ease comp/financials, pull Chess in, detail Day 3</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="10" t="n">
+      <c r="A110" s="12" t="n">
         <v>107</v>
       </c>
-      <c r="B110" s="10" t="inlineStr">
+      <c r="B110" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:13</t>
         </is>
       </c>
-      <c r="C110" s="10" t="inlineStr">
+      <c r="C110" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D110" s="12" t="inlineStr">
+      <c r="D110" s="14" t="inlineStr">
         <is>
           <t>Correct for Magic's departure + add weekend primer</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="10" t="n">
+      <c r="A111" s="12" t="n">
         <v>108</v>
       </c>
-      <c r="B111" s="10" t="inlineStr">
+      <c r="B111" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:24</t>
         </is>
       </c>
-      <c r="C111" s="10" t="inlineStr">
+      <c r="C111" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D111" s="12" t="inlineStr">
+      <c r="D111" s="14" t="inlineStr">
         <is>
           <t>Weekend primer: Lotus/itachi = consultants, Odi runs X, + Saturday Space, challenge-to-play, example posts</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="10" t="n">
+      <c r="A112" s="12" t="n">
         <v>109</v>
       </c>
-      <c r="B112" s="10" t="inlineStr">
+      <c r="B112" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:35</t>
         </is>
       </c>
-      <c r="C112" s="10" t="inlineStr">
+      <c r="C112" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D112" s="12" t="inlineStr">
+      <c r="D112" s="14" t="inlineStr">
         <is>
           <t>Scrub all 'bundle' mentions; reframe Bao/nerd + Lotus/itachi as outside (not team)</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="10" t="n">
+      <c r="A113" s="12" t="n">
         <v>110</v>
       </c>
-      <c r="B113" s="10" t="inlineStr">
+      <c r="B113" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:47</t>
         </is>
       </c>
-      <c r="C113" s="10" t="inlineStr">
+      <c r="C113" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D113" s="12" t="inlineStr">
+      <c r="D113" s="14" t="inlineStr">
         <is>
           <t>Add X Space talking-points cheat sheet (Sat) — beats, soundbites, hard-Q answers, guardrails</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="10" t="n">
+      <c r="A114" s="12" t="n">
         <v>111</v>
       </c>
-      <c r="B114" s="10" t="inlineStr">
+      <c r="B114" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:51</t>
         </is>
       </c>
-      <c r="C114" s="10" t="inlineStr">
+      <c r="C114" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D114" s="12" t="inlineStr">
+      <c r="D114" s="14" t="inlineStr">
         <is>
           <t>Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6bf157372e19db43bc75fda	2026-06-26T15:58:55-04:00	ruby-trivia	docs(web3): independent legal/regulatory research report</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="10" t="n">
+      <c r="A115" s="12" t="n">
         <v>112</v>
       </c>
-      <c r="B115" s="10" t="inlineStr">
+      <c r="B115" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 10:59</t>
         </is>
       </c>
-      <c r="C115" s="10" t="inlineStr">
+      <c r="C115" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D115" s="12" t="inlineStr">
+      <c r="D115" s="14" t="inlineStr">
         <is>
           <t>Strip theme banner; landing page = just the team + weekend links (nothing above)</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="10" t="n">
+      <c r="A116" s="12" t="n">
         <v>113</v>
       </c>
-      <c r="B116" s="10" t="inlineStr">
+      <c r="B116" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 11:04</t>
         </is>
       </c>
-      <c r="C116" s="10" t="inlineStr">
+      <c r="C116" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D116" s="12" t="inlineStr">
+      <c r="D116" s="14" t="inlineStr">
         <is>
           <t>Weekend page: put the actionable plan back (X post examples, thread, challenge copy, Space) — minus internal-only bits</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="10" t="n">
+      <c r="A117" s="12" t="n">
         <v>114</v>
       </c>
-      <c r="B117" s="10" t="inlineStr">
+      <c r="B117" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 11:09</t>
         </is>
       </c>
-      <c r="C117" s="10" t="inlineStr">
+      <c r="C117" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D117" s="12" t="inlineStr">
+      <c r="D117" s="14" t="inlineStr">
         <is>
           <t>Add public FAQ (hard questions, cleaned) + link from landing</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="10" t="n">
+      <c r="A118" s="12" t="n">
         <v>115</v>
       </c>
-      <c r="B118" s="10" t="inlineStr">
+      <c r="B118" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 11:16</t>
         </is>
       </c>
-      <c r="C118" s="10" t="inlineStr">
+      <c r="C118" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D118" s="12" t="inlineStr">
+      <c r="D118" s="14" t="inlineStr">
         <is>
           <t>Team: Dutch + Odi are the two-person core, tied across everything (not split by frontend/backend)</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="10" t="n">
+      <c r="A119" s="12" t="n">
         <v>116</v>
       </c>
-      <c r="B119" s="10" t="inlineStr">
+      <c r="B119" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 11:23</t>
         </is>
       </c>
-      <c r="C119" s="10" t="inlineStr">
+      <c r="C119" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D119" s="12" t="inlineStr">
+      <c r="D119" s="14" t="inlineStr">
         <is>
           <t>Clarify: posts are examples to work from (not post-as-is); designate X = Odi; community = TG (Destiny), not X</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="10" t="n">
+      <c r="A120" s="12" t="n">
         <v>117</v>
       </c>
-      <c r="B120" s="10" t="inlineStr">
+      <c r="B120" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 11:39</t>
         </is>
       </c>
-      <c r="C120" s="10" t="inlineStr">
+      <c r="C120" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D120" s="12" t="inlineStr">
+      <c r="D120" s="14" t="inlineStr">
         <is>
           <t>Sync private docs to handbook: Dutch+Odi tied across everything; toolkit = examples to work from (not canned posts)</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="10" t="n">
+      <c r="A121" s="12" t="n">
         <v>118</v>
       </c>
-      <c r="B121" s="10" t="inlineStr">
+      <c r="B121" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 12:51</t>
         </is>
       </c>
-      <c r="C121" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D121" s="12" t="inlineStr">
+      <c r="C121" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
         <is>
           <t>feat(bot): /stats — lifetime avg points per question &amp; per round</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="10" t="n">
+      <c r="A122" s="12" t="n">
         <v>119</v>
       </c>
-      <c r="B122" s="10" t="inlineStr">
+      <c r="B122" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 13:44</t>
         </is>
       </c>
-      <c r="C122" s="10" t="inlineStr">
+      <c r="C122" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D122" s="12" t="inlineStr">
+      <c r="D122" s="14" t="inlineStr">
         <is>
           <t>Titles + decision structure + capacity/slow-roll across planning set</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="10" t="n">
+      <c r="A123" s="12" t="n">
         <v>120</v>
       </c>
-      <c r="B123" s="10" t="inlineStr">
+      <c r="B123" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 13:45</t>
         </is>
       </c>
-      <c r="C123" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D123" s="12" t="inlineStr">
+      <c r="C123" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
         <is>
           <t>feat(stats): efficiency averages across all telegram modes + web profile</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="10" t="n">
+      <c r="A124" s="12" t="n">
         <v>121</v>
       </c>
-      <c r="B124" s="10" t="inlineStr">
+      <c r="B124" s="12" t="inlineStr">
         <is>
           <t>2026-06-26 15:53</t>
         </is>
       </c>
-      <c r="C124" s="10" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D124" s="12" t="inlineStr">
+      <c r="C124" s="12" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
         <is>
           <t>docs(web3): branch for tokenomics/NFT work + compliance guardrails</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="10" t="n">
+      <c r="A125" s="12" t="n">
         <v>122</v>
       </c>
-      <c r="B125" s="10" t="inlineStr">
+      <c r="B125" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 19:04</t>
         </is>
       </c>
-      <c r="C125" s="10" t="inlineStr">
+      <c r="C125" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D125" s="12" t="inlineStr">
+      <c r="D125" s="14" t="inlineStr">
         <is>
           <t>Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel web2/web3, risk-parity control)</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="10" t="n">
+      <c r="A126" s="12" t="n">
         <v>123</v>
       </c>
-      <c r="B126" s="10" t="inlineStr">
+      <c r="B126" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 19:10</t>
         </is>
       </c>
-      <c r="C126" s="10" t="inlineStr">
+      <c r="C126" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D126" s="12" t="inlineStr">
+      <c r="D126" s="14" t="inlineStr">
         <is>
           <t>Add 07: tax &amp; legal/regulatory research (cited) for the governance structure</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="10" t="n">
+      <c r="A127" s="12" t="n">
         <v>124</v>
       </c>
-      <c r="B127" s="10" t="inlineStr">
+      <c r="B127" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 19:17</t>
         </is>
       </c>
-      <c r="C127" s="10" t="inlineStr">
+      <c r="C127" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D127" s="12" t="inlineStr">
+      <c r="D127" s="14" t="inlineStr">
         <is>
           <t>Add 08: latest 2025-26 statutes + how-others-do-it playbooks + right-sized recommended path</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="10" t="n">
+      <c r="A128" s="12" t="n">
         <v>125</v>
       </c>
-      <c r="B128" s="10" t="inlineStr">
+      <c r="B128" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 20:05</t>
         </is>
       </c>
-      <c r="C128" s="10" t="inlineStr">
+      <c r="C128" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D128" s="12" t="inlineStr">
+      <c r="D128" s="14" t="inlineStr">
         <is>
           <t>Add browsable docs hub (README front page) + S-corp analysis across 06/07/08</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="10" t="n">
+      <c r="A129" s="12" t="n">
         <v>126</v>
       </c>
-      <c r="B129" s="10" t="inlineStr">
+      <c r="B129" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 20:22</t>
         </is>
       </c>
-      <c r="C129" s="10" t="inlineStr">
+      <c r="C129" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D129" s="12" t="inlineStr">
+      <c r="D129" s="14" t="inlineStr">
         <is>
           <t>Add founder/operator compensation working proposal (24h counter window) to 06; thread through 07/08/README</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="10" t="n">
+      <c r="A130" s="12" t="n">
         <v>127</v>
       </c>
-      <c r="B130" s="10" t="inlineStr">
+      <c r="B130" s="12" t="inlineStr">
         <is>
           <t>2026-06-29 20:50</t>
         </is>
       </c>
-      <c r="C130" s="10" t="inlineStr">
+      <c r="C130" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D130" s="12" t="inlineStr">
+      <c r="D130" s="14" t="inlineStr">
         <is>
           <t>Comp: operator draw is CAPPED at a fair daily wage (excess stays in treasury)</t>
         </is>
@@ -3865,28 +3888,28 @@
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>• Hours from GitHub commit timestamps. Floor = git-hours method (&gt;2h gap=new session, +2h ramp). Realistic = active-day method weighted by commit intensity (heaviest day ~16h, normal active day ~8h).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>• All commits under 'dutch &lt;dutchiono@gmail.com&gt;' / GitHub 'dutchiono' across all Ruby repos. Other contributors excluded.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>• Date range 2026-05-29 to 2026-06-29; 13 active days; 127 commits.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>• Amount paid to date: $350. Three rate scenarios: $10, $50, $150/hr.</t>
         </is>

</xml_diff>

<commit_message>
Fix tables: real HTML table (markdown tables weren't rendering); drop invoice framing; one clean table + receipts
</commit_message>
<xml_diff>
--- a/Dutch-Ruby-Comp-Claim.xlsx
+++ b/Dutch-Ruby-Comp-Claim.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bill &amp; Bid" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hours &amp; Rates" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hours by Day" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What was built" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commit Log" sheetId="4" state="visible" r:id="rId4"/>
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,10 +38,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -93,16 +89,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -492,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -505,7 +499,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ruby Trivia — Bill &amp; Bid (Dutch / dutchiono)</t>
+          <t>Ruby Trivia — Hours &amp; Rates (Dutch / dutchiono)</t>
         </is>
       </c>
     </row>
@@ -567,103 +561,93 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>AMOUNT DUE  (106 hrs × $50 agreed − $350 paid)</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>4950</v>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>The hours at three rates (minus $350 paid):</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Owed</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>BID — the same hours at three rates</t>
-        </is>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>$10/hr</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>106</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>710</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Hours</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Owed</t>
-        </is>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>$25/hr</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>106</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>2650</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>2300</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>$10/hr</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>$50/hr</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
         <v>106</v>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>1060</v>
-      </c>
-      <c r="D15" s="10" t="n">
+      <c r="C15" s="8" t="n">
+        <v>5300</v>
+      </c>
+      <c r="D15" s="8" t="n">
         <v>350</v>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>$25/hr</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="n">
-        <v>106</v>
-      </c>
-      <c r="C16" s="10" t="n">
-        <v>2650</v>
-      </c>
-      <c r="D16" s="10" t="n">
-        <v>350</v>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>$50/hr</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>106</v>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>5300</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>350</v>
-      </c>
-      <c r="E17" s="11" t="n">
+      <c r="E15" s="9" t="n">
         <v>4950</v>
       </c>
     </row>
@@ -699,458 +683,458 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Commits</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Hrs</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>@ $10</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>@ $25</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>@ $50</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Repos / sample work</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="G4" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ru</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">ruby-trivia — untracked files on iono/games-production: dc3e01f Archive iono games production </t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="G9" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>ruby-labs — Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="G10" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="G11" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="G12" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — CI: use plain bun install (lockfile drifts across bun versions) + resync bun.loc</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>ruby-trivia — fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G14" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia — Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcb</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="G15" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing, ruby-trivia, ruby-trivia-handbook — Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="G16" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>ruby-marketing — Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel we</t>
         </is>
@@ -1169,13 +1153,13 @@
       <c r="D17" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="13" t="n">
         <v>1060</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="13" t="n">
         <v>2650</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="13" t="n">
         <v>5300</v>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1205,70 +1189,70 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>• Trivia PWA — daily quiz, practice, friend challenges, leaderboards, streaks, ranks/badges, 4 languages, installable</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>• Live multiplayer — realtime WebSocket lobbies, matchmaking, graceful reconnect</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>• Backend &amp; API — Hono/Bun server, auth/registration, game logic, SQLite→MariaDB migration + SQL translation</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>• Web3 holder layer — Solana wallet connect, holder verification, perks (multiplier, holders-only leaderboard, cosmetics)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>• On-chain / contracts — contract suite, result-signer seam, token integration</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>• Telegram bot gateway — in-chat trivia, stateless solo play, /stats</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>• Production infra / DevOps — multi-container, nginx, MariaDB, deploy scripts, live incident response</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>• App-store repackaging — Capacitor + multi-store editions</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>• Token launch support &amp; ops — Solana/Pump.fun launch, splash/CA, coordination</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>• Educational variant — ruby-trivia-classroom</t>
         </is>
@@ -1302,2562 +1286,2562 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Date / time</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Repo</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>2026-05-29 22:58</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>add magidir28fce635ba862adae07e53c3f4f9d0c7a4bfaeac	2026-06-25T00:50:18-04:00	ruby-labs	feat: sync latest marketing landing from ruby-trivia + i18n; purge bushleague</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 10:58</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Ship Ruby Trivia classroom hub with library-themed UI for bushleague.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:41</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Fix shelf book launches, clay UI, classroom sounds and haptics.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Mobile-first layout and full main-repo trivia parity.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:44</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Fix deploy script staging cleanup on Windows.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:47</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Add GitHub Actions auto-deploy to classroom.bushleague.xyz on push to master.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:49</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Fix GitHub Actions deploy SSH key and scp paths.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:51</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Fix CI deploy rsync when scp nests files under dist/.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 22:56</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Remove Class from header; rename nav to Lessons.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:00</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Boost clay depth and sounds; drop fake leaderboard names.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:03</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Replace open Create with curated quiz sets; drop unsigned custom questions.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:04</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Fix nav sounds: play on tab click inside user gesture.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:05</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Stop defaulting player name to Ruby; clear persisted Ruby names.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:07</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Block Ruby as player name; no anonymous leaderboard rows.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:08</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Add preferred Ruby Trivia logo to header.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n">
+      <c r="A19" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:10</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Omit unnamed players from scoreboards; document backend contract.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:12</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Put Trivia above Lessons in nav.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>2026-06-16 23:14</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Remove duplicate hero logo; use downloaded sound files for cues.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>2026-06-17 22:12</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Ship Play live multiplayer, trivia-first nav, and content curation policy.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>2026-06-17 22:15</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Fix deploy script line endings and static upload cleanup.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 17:15</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Split Ruby Labs hub and Ruby Games app with dual-site deploy.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 17:28</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Restructure mobile nav around Games hub and add Odie's Car.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>2026-06-18 22:45</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Add Bush League clay dress kit and apply theme to app shell.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n">
+      <c r="A27" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 14:33</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 14:34</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Add single-repo workflow doc after consolidating on ruby-high/ruby-trivia.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n">
+      <c r="A29" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>index on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>2026-06-19 17:47</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>untracked files on iono/games-production: dc3e01f Archive iono games production fork (WS multiplayer, Games hub, dress-kit docs).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n">
+      <c r="A31" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>Initial Ruby Labs marketing site for ruby-high org.44203a64ebaf018ac116e4a8b2b1e675af6ce46b	2026-06-25T04:50:33-04:00	dutchiono-ruby-trivia	feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n">
+      <c r="A32" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>2026-06-20 20:21</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>ruby-labs</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>Ignore TypeScript build info files.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n">
+      <c r="A33" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>2026-06-21 02:51</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Add mobile-first nav, in-app docs, and demo deploy tooling on clay reskin.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:23</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Fix clay content contrast: scope sidebar crew colors and darken muted text.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="n">
+      <c r="A35" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:27</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Add auth intent persistence and fix live room invite flow.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n">
+      <c r="A36" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:33</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Harden anotherone deploy: exclude server node_modules from upload.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="n">
+      <c r="A37" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 13:37</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>Fix unreadable theme-option buttons on clay cards in dark mode.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 14:45</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>Add side dock rail, RUBYSQUARE header mark, and clay contrast fixes.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="n">
+      <c r="A39" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>2026-06-22 21:22</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>Remove third-party studio branding and add session handoff doc.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n">
+      <c r="A40" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 06:22</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>Document single-branch workflow; rename archive branch.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="n">
+      <c r="A41" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D41" s="14" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="n">
+      <c r="A42" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 08:45</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Wire sensory audio and haptics into trivia nav and quiz flows.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="n">
+      <c r="A43" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 10:52</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>Add ring-aling bell sound alongside sensory MP3 cues.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="n">
+      <c r="A45" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:22</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D45" s="14" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>Use MP3-only sensory assets from Audacity exports.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:29</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D46" s="14" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>Add on-chain scaffold, chain signer API, brand assets, and trivia data.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="n">
+      <c r="A47" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 11:40</t>
         </is>
       </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D47" s="14" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>Show Ruby Trivia logo in minimized mobile header chrome.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n">
+      <c r="A48" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 12:09</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>Fix minimized mobile header: slim RUBYSQUARE pill, no side rail.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="n">
+      <c r="A49" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 12:29</t>
         </is>
       </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D49" s="14" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Route nav sounds: zipper on top dock, page on bottom subnav, paper on ranks.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="n">
+      <c r="A50" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 15:56</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D50" s="14" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>Refactor trivia navigation: bottom nav, mode nav, games layout</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="n">
+      <c r="A51" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 18:26</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D51" s="14" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>Fix unreadable secondary buttons on cream modals</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="n">
+      <c r="A52" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 19:46</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D52" s="14" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>Fix missing desktop nav rail in authenticated layout</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="12" t="n">
+      <c r="A53" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:02</t>
         </is>
       </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>Warm blue chrome to clay palette + add Docs to desktop nav</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n">
+      <c r="A54" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:07</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D54" s="14" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>Reskin splash CTA from blue to clay orange</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="n">
+      <c r="A55" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:09</t>
         </is>
       </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>Warm active language-picker chip to clay orange</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n">
+      <c r="A56" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B56" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:12</t>
         </is>
       </c>
-      <c r="C56" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D56" s="14" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>Warm language-button focus outline to clay orange</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B57" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:34</t>
         </is>
       </c>
-      <c r="C57" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>Public /docs route, clay answer buttons, warm crew links</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="n">
+      <c r="A58" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B58" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 20:43</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D58" s="14" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>Fix production DB corruption: stop deploy from clobbering the live SQLite db</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="12" t="n">
+      <c r="A59" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B59" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:06</t>
         </is>
       </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>Add PR CI: build + chain tests</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
+      <c r="A60" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B60" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:08</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>CI: use plain bun install (lockfile drifts across bun versions) + resync bun.lock</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="n">
+      <c r="A61" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B61" s="10" t="inlineStr">
         <is>
           <t>2026-06-23 21:27</t>
         </is>
       </c>
-      <c r="C61" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>Add full social meta, PWA manifest, and app/Farcaster embeds</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n">
+      <c r="A62" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="B62" s="12" t="inlineStr">
+      <c r="B62" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:00</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>i18n: re-translate zh UI (replace machine-slop) + complete es gaps</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="n">
+      <c r="A63" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B63" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:07</t>
         </is>
       </c>
-      <c r="C63" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>i18n: add French (fr) locale</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n">
+      <c r="A64" s="10" t="n">
         <v>61</v>
       </c>
-      <c r="B64" s="12" t="inlineStr">
+      <c r="B64" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:18</t>
         </is>
       </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>Fix build: stop hardcoding /srv/www as vite outDir</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="n">
+      <c r="A65" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B65" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:21</t>
         </is>
       </c>
-      <c r="C65" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>i18n: accept fr in server locale enums (register, set-locale, admin, questions)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="n">
+      <c r="A66" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="B66" s="12" t="inlineStr">
+      <c r="B66" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 08:38</t>
         </is>
       </c>
-      <c r="C66" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D66" s="14" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
         <is>
           <t>docs: thorough Privacy Policy + Terms of Use (token/no-returns, liability)</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="12" t="n">
+      <c r="A67" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B67" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 09:23</t>
         </is>
       </c>
-      <c r="C67" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D67" s="14" t="inlineStr">
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>docs: make web3 forward-looking for no-web3 launch; stash full token terms</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="n">
+      <c r="A68" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B68" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 09:57</t>
         </is>
       </c>
-      <c r="C68" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
         <is>
           <t>ci: skip bushleague/labs demo deploy when DEPLOY_SSH_KEY is unset</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="12" t="n">
+      <c r="A69" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B69" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 10:32</t>
         </is>
       </c>
-      <c r="C69" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>docs: add pre-launch review (findings for lead dev / legal / ops)</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="n">
+      <c r="A70" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B70" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 11:49</t>
         </is>
       </c>
-      <c r="C70" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
         <is>
           <t>fix(server): await migration async gaps in register + trivia/rush-hour answer paths</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="12" t="n">
+      <c r="A71" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B71" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:08</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
         <is>
           <t>[WIP] async-correctness sweep (NOT deployable yet — server tree does not compile clean)</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="n">
+      <c r="A72" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="B72" s="12" t="inlineStr">
+      <c r="B72" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:53</t>
         </is>
       </c>
-      <c r="C72" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D72" s="14" t="inlineStr">
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>Fix MariaDB-migration async/await gaps across the server (full sweep)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="n">
+      <c r="A73" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="B73" s="12" t="inlineStr">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 12:57</t>
         </is>
       </c>
-      <c r="C73" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D73" s="14" t="inlineStr">
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>ci: exclude legacy server/src from server typecheck gate</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="n">
+      <c r="A74" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="B74" s="12" t="inlineStr">
+      <c r="B74" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 14:03</t>
         </is>
       </c>
-      <c r="C74" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>docs(roadmap): add staking to the deferred token terms (yield + partner undecided)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="12" t="n">
+      <c r="A75" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 14:37</t>
         </is>
       </c>
-      <c r="C75" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D75" s="14" t="inlineStr">
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>ui: fix guest CTA card spacing, surface docs on desktop, add placeholder CA pill</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="n">
+      <c r="A76" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="B76" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 15:17</t>
         </is>
       </c>
-      <c r="C76" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
         <is>
           <t>fix: don't blank the app when /api/games returns a non-array</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="12" t="n">
+      <c r="A77" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="B77" s="12" t="inlineStr">
+      <c r="B77" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 16:43</t>
         </is>
       </c>
-      <c r="C77" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
         <is>
           <t>docs: add Roadmap page + purge bushleague from user-facing copy</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="n">
+      <c r="A78" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="B78" s="12" t="inlineStr">
+      <c r="B78" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 16:57</t>
         </is>
       </c>
-      <c r="C78" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D78" s="14" t="inlineStr">
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
         <is>
           <t>chore: purge bushleague from everything in code (relic — it's only a host name)</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="12" t="n">
+      <c r="A79" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="B79" s="12" t="inlineStr">
+      <c r="B79" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:02</t>
         </is>
       </c>
-      <c r="C79" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D79" s="14" t="inlineStr">
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
         <is>
           <t>chore: set official token contract address (CA pill)</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="12" t="n">
+      <c r="A80" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="12" t="inlineStr">
+      <c r="B80" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:16</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D80" s="14" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
         <is>
           <t>docs: reconcile chain references to Solana (token moved from BSC)</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="12" t="n">
+      <c r="A81" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="B81" s="12" t="inlineStr">
+      <c r="B81" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 17:56</t>
         </is>
       </c>
-      <c r="C81" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D81" s="14" t="inlineStr">
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D81" s="12" t="inlineStr">
         <is>
           <t>docs: full Roadmap (vision, Now / 30-day / 60-day / Beyond)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="12" t="n">
+      <c r="A82" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="B82" s="12" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:04</t>
         </is>
       </c>
-      <c r="C82" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D82" s="14" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D82" s="12" t="inlineStr">
         <is>
           <t>fix: trivia sounds = beeps/boops only + tighten quiz spacing</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="12" t="n">
+      <c r="A83" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="B83" s="12" t="inlineStr">
+      <c r="B83" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:41</t>
         </is>
       </c>
-      <c r="C83" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D83" s="14" t="inlineStr">
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
         <is>
           <t>feat(web3): Solana holder-perks layer (web3.ruby-trivia.com)</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="n">
+      <c r="A84" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="B84" s="12" t="inlineStr">
+      <c r="B84" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 19:49</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
         <is>
           <t>docs: prod backend handoff — master&lt;-&gt;MariaDB divergence (for Odi)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="12" t="n">
+      <c r="A85" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="B85" s="12" t="inlineStr">
+      <c r="B85" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 20:59</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D85" s="14" t="inlineStr">
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
         <is>
           <t>feat(web3 UI): wallet connect in bottom nav + polish (for Odi to integrate)</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="12" t="n">
+      <c r="A86" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="B86" s="12" t="inlineStr">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 22:50</t>
         </is>
       </c>
-      <c r="C86" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D86" s="14" t="inlineStr">
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
         <is>
           <t>fix(web3 demo): branding purge, guest mobile nav, emoji PFP, daily-reward + desktop wallet</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="12" t="n">
+      <c r="A87" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="B87" s="12" t="inlineStr">
+      <c r="B87" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:17</t>
         </is>
       </c>
-      <c r="C87" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D87" s="14" t="inlineStr">
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
         <is>
           <t>fix(web3): show wallet Connect in guest mode (sidebar + bottom nav)</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="12" t="n">
+      <c r="A88" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="B88" s="12" t="inlineStr">
+      <c r="B88" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:24</t>
         </is>
       </c>
-      <c r="C88" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D88" s="14" t="inlineStr">
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
         <is>
           <t>fix(nav): guest desktop sidebar 1:1 with mobile bottom nav</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="12" t="n">
+      <c r="A89" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="B89" s="12" t="inlineStr">
+      <c r="B89" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:26</t>
         </is>
       </c>
-      <c r="C89" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D89" s="14" t="inlineStr">
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
         <is>
           <t>fix(i18n): add missing quiz.todaysQuiz key (was rendering raw "quiz.todaysQuiz")</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="12" t="n">
+      <c r="A90" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="B90" s="12" t="inlineStr">
+      <c r="B90" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:32</t>
         </is>
       </c>
-      <c r="C90" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D90" s="14" t="inlineStr">
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>i18n(web3): translate wallet-modal strings into all locales</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="12" t="n">
+      <c r="A91" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="B91" s="12" t="inlineStr">
+      <c r="B91" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:40</t>
         </is>
       </c>
-      <c r="C91" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
         <is>
           <t>fix(i18n): translate practice-topic category labels</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="12" t="n">
+      <c r="A92" s="10" t="n">
         <v>89</v>
       </c>
-      <c r="B92" s="12" t="inlineStr">
+      <c r="B92" s="10" t="inlineStr">
         <is>
           <t>2026-06-24 23:48</t>
         </is>
       </c>
-      <c r="C92" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
         <is>
           <t>fix(guest): restore Sign in / Create account CTA on guest profile (mobile login)</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="12" t="n">
+      <c r="A93" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="B93" s="12" t="inlineStr">
+      <c r="B93" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 00:08</t>
         </is>
       </c>
-      <c r="C93" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D93" s="14" t="inlineStr">
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
         <is>
           <t>fix(deploy): kill labs subdomain — labs.ruby-trivia.com → www.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="12" t="n">
+      <c r="A94" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="B94" s="12" t="inlineStr">
+      <c r="B94" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 00:28</t>
         </is>
       </c>
-      <c r="C94" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D94" s="14" t="inlineStr">
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
         <is>
           <t>fix(deploy): actually build + ship the web3 bundle to web3.ruby-trivia.com</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="12" t="n">
+      <c r="A95" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="B95" s="12" t="inlineStr">
+      <c r="B95" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 01:10</t>
         </is>
       </c>
-      <c r="C95" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
         <is>
           <t>fix(web3): error-boundary the wallet nav button so it can't take down the nav</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="12" t="n">
+      <c r="A96" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="12" t="inlineStr">
+      <c r="B96" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 02:21</t>
         </is>
       </c>
-      <c r="C96" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
         <is>
           <t>docs: fix stale BNB Smart Chain refs (token is live on Solana)</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="12" t="n">
+      <c r="A97" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="B97" s="12" t="inlineStr">
+      <c r="B97" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 02:26</t>
         </is>
       </c>
-      <c r="C97" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
         <is>
           <t>docs: token ticker is $TRIVIA, not RUBY (Ruby Trivia is the game)</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="12" t="n">
+      <c r="A98" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="B98" s="12" t="inlineStr">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 04:50</t>
         </is>
       </c>
-      <c r="C98" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D98" s="14" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D98" s="12" t="inlineStr">
         <is>
           <t>feat(splash): show token CA pill on the welcome/language screen</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="12" t="n">
+      <c r="A99" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="B99" s="12" t="inlineStr">
+      <c r="B99" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C99" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D99" s="14" t="inlineStr">
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="12" t="n">
+      <c r="A100" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="B100" s="12" t="inlineStr">
+      <c r="B100" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 13:26</t>
         </is>
       </c>
-      <c r="C100" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D100" s="14" t="inlineStr">
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D100" s="12" t="inlineStr">
         <is>
           <t>fix(db): translate SQLite ON CONFLICT upsert to MariaDB ON DUPLICATE KEY</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="12" t="n">
+      <c r="A101" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="B101" s="12" t="inlineStr">
+      <c r="B101" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 15:49</t>
         </is>
       </c>
-      <c r="C101" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D101" s="14" t="inlineStr">
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr">
         <is>
           <t>fix(web2): hide token CA pill in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="12" t="n">
+      <c r="A102" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="B102" s="12" t="inlineStr">
+      <c r="B102" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 15:53</t>
         </is>
       </c>
-      <c r="C102" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D102" s="14" t="inlineStr">
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
         <is>
           <t>fix(web2): hide tokenomics docs article in web2/store builds</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="12" t="n">
+      <c r="A103" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="B103" s="12" t="inlineStr">
+      <c r="B103" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 16:39</t>
         </is>
       </c>
-      <c r="C103" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D103" s="14" t="inlineStr">
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
         <is>
           <t>feat(store): ship native app as free v1 (no subscribe stub)</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="12" t="n">
+      <c r="A104" s="10" t="n">
         <v>101</v>
       </c>
-      <c r="B104" s="12" t="inlineStr">
+      <c r="B104" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 16:47</t>
         </is>
       </c>
-      <c r="C104" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D104" s="14" t="inlineStr">
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
         <is>
           <t>feat(live): resilient WS reconnect — backoff, auto-rejoin, graceful fail</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="12" t="n">
+      <c r="A105" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="B105" s="12" t="inlineStr">
+      <c r="B105" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 17:44</t>
         </is>
       </c>
-      <c r="C105" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D105" s="14" t="inlineStr">
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="inlineStr">
         <is>
           <t>docs: app-store distribution plan + session handoff</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="12" t="n">
+      <c r="A106" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="B106" s="12" t="inlineStr">
+      <c r="B106" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 18:12</t>
         </is>
       </c>
-      <c r="C106" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D106" s="14" t="inlineStr">
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D106" s="12" t="inlineStr">
         <is>
           <t>feat(live): broadcast stage view of live trivia rounds (P0)</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="12" t="n">
+      <c r="A107" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="B107" s="12" t="inlineStr">
+      <c r="B107" s="10" t="inlineStr">
         <is>
           <t>2026-06-25 18:22</t>
         </is>
       </c>
-      <c r="C107" s="12" t="inlineStr">
+      <c r="C107" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D107" s="14" t="inlineStr">
+      <c r="D107" s="12" t="inlineStr">
         <is>
           <t>Add X Space outline (2026-06-25) + repo README8f80a5bf9ca556506fb5b84005a0be9dcbd610a5	2026-06-26T13:45:01-04:00	ruby-trivia-handbook	Handbook: add public titles (Dutch = lead dev, Odi = lead marketing); both doing both</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="12" t="n">
+      <c r="A108" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="B108" s="12" t="inlineStr">
+      <c r="B108" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 09:37</t>
         </is>
       </c>
-      <c r="C108" s="12" t="inlineStr">
+      <c r="C108" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D108" s="14" t="inlineStr">
+      <c r="D108" s="12" t="inlineStr">
         <is>
           <t>Add manager planning set: state-of-project, idea bank, roadmap, 1/3/7/14/30-day deliverables, team instructions, risks/ops</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="12" t="n">
+      <c r="A109" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="B109" s="12" t="inlineStr">
+      <c r="B109" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:00</t>
         </is>
       </c>
-      <c r="C109" s="12" t="inlineStr">
+      <c r="C109" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D109" s="14" t="inlineStr">
+      <c r="D109" s="12" t="inlineStr">
         <is>
           <t>Sensitivity pass: soften ownership language, ease comp/financials, pull Chess in, detail Day 3</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="12" t="n">
+      <c r="A110" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="B110" s="12" t="inlineStr">
+      <c r="B110" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:13</t>
         </is>
       </c>
-      <c r="C110" s="12" t="inlineStr">
+      <c r="C110" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D110" s="14" t="inlineStr">
+      <c r="D110" s="12" t="inlineStr">
         <is>
           <t>Correct for Magic's departure + add weekend primer</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="12" t="n">
+      <c r="A111" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="B111" s="12" t="inlineStr">
+      <c r="B111" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:24</t>
         </is>
       </c>
-      <c r="C111" s="12" t="inlineStr">
+      <c r="C111" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D111" s="14" t="inlineStr">
+      <c r="D111" s="12" t="inlineStr">
         <is>
           <t>Weekend primer: Lotus/itachi = consultants, Odi runs X, + Saturday Space, challenge-to-play, example posts</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="12" t="n">
+      <c r="A112" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="B112" s="12" t="inlineStr">
+      <c r="B112" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:35</t>
         </is>
       </c>
-      <c r="C112" s="12" t="inlineStr">
+      <c r="C112" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D112" s="14" t="inlineStr">
+      <c r="D112" s="12" t="inlineStr">
         <is>
           <t>Scrub all 'bundle' mentions; reframe Bao/nerd + Lotus/itachi as outside (not team)</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="12" t="n">
+      <c r="A113" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="B113" s="12" t="inlineStr">
+      <c r="B113" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:47</t>
         </is>
       </c>
-      <c r="C113" s="12" t="inlineStr">
+      <c r="C113" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D113" s="14" t="inlineStr">
+      <c r="D113" s="12" t="inlineStr">
         <is>
           <t>Add X Space talking-points cheat sheet (Sat) — beats, soundbites, hard-Q answers, guardrails</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="12" t="n">
+      <c r="A114" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="B114" s="12" t="inlineStr">
+      <c r="B114" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:51</t>
         </is>
       </c>
-      <c r="C114" s="12" t="inlineStr">
+      <c r="C114" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D114" s="14" t="inlineStr">
+      <c r="D114" s="12" t="inlineStr">
         <is>
           <t>Public handbook: how we work + this weekend (community-facing)2bf7eff9e5d10e38f6bf157372e19db43bc75fda	2026-06-26T15:58:55-04:00	ruby-trivia	docs(web3): independent legal/regulatory research report</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="12" t="n">
+      <c r="A115" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="B115" s="12" t="inlineStr">
+      <c r="B115" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 10:59</t>
         </is>
       </c>
-      <c r="C115" s="12" t="inlineStr">
+      <c r="C115" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D115" s="14" t="inlineStr">
+      <c r="D115" s="12" t="inlineStr">
         <is>
           <t>Strip theme banner; landing page = just the team + weekend links (nothing above)</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="12" t="n">
+      <c r="A116" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="B116" s="12" t="inlineStr">
+      <c r="B116" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:04</t>
         </is>
       </c>
-      <c r="C116" s="12" t="inlineStr">
+      <c r="C116" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D116" s="14" t="inlineStr">
+      <c r="D116" s="12" t="inlineStr">
         <is>
           <t>Weekend page: put the actionable plan back (X post examples, thread, challenge copy, Space) — minus internal-only bits</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="12" t="n">
+      <c r="A117" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="B117" s="12" t="inlineStr">
+      <c r="B117" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:09</t>
         </is>
       </c>
-      <c r="C117" s="12" t="inlineStr">
+      <c r="C117" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D117" s="14" t="inlineStr">
+      <c r="D117" s="12" t="inlineStr">
         <is>
           <t>Add public FAQ (hard questions, cleaned) + link from landing</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="12" t="n">
+      <c r="A118" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="B118" s="12" t="inlineStr">
+      <c r="B118" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:16</t>
         </is>
       </c>
-      <c r="C118" s="12" t="inlineStr">
+      <c r="C118" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D118" s="14" t="inlineStr">
+      <c r="D118" s="12" t="inlineStr">
         <is>
           <t>Team: Dutch + Odi are the two-person core, tied across everything (not split by frontend/backend)</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="12" t="n">
+      <c r="A119" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="B119" s="12" t="inlineStr">
+      <c r="B119" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:23</t>
         </is>
       </c>
-      <c r="C119" s="12" t="inlineStr">
+      <c r="C119" s="10" t="inlineStr">
         <is>
           <t>ruby-trivia-handbook</t>
         </is>
       </c>
-      <c r="D119" s="14" t="inlineStr">
+      <c r="D119" s="12" t="inlineStr">
         <is>
           <t>Clarify: posts are examples to work from (not post-as-is); designate X = Odi; community = TG (Destiny), not X</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="12" t="n">
+      <c r="A120" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="B120" s="12" t="inlineStr">
+      <c r="B120" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 11:39</t>
         </is>
       </c>
-      <c r="C120" s="12" t="inlineStr">
+      <c r="C120" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D120" s="14" t="inlineStr">
+      <c r="D120" s="12" t="inlineStr">
         <is>
           <t>Sync private docs to handbook: Dutch+Odi tied across everything; toolkit = examples to work from (not canned posts)</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="12" t="n">
+      <c r="A121" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="B121" s="12" t="inlineStr">
+      <c r="B121" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 12:51</t>
         </is>
       </c>
-      <c r="C121" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D121" s="14" t="inlineStr">
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="inlineStr">
         <is>
           <t>feat(bot): /stats — lifetime avg points per question &amp; per round</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="12" t="n">
+      <c r="A122" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="B122" s="12" t="inlineStr">
+      <c r="B122" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 13:44</t>
         </is>
       </c>
-      <c r="C122" s="12" t="inlineStr">
+      <c r="C122" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D122" s="14" t="inlineStr">
+      <c r="D122" s="12" t="inlineStr">
         <is>
           <t>Titles + decision structure + capacity/slow-roll across planning set</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="12" t="n">
+      <c r="A123" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="B123" s="12" t="inlineStr">
+      <c r="B123" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 13:45</t>
         </is>
       </c>
-      <c r="C123" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D123" s="14" t="inlineStr">
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="inlineStr">
         <is>
           <t>feat(stats): efficiency averages across all telegram modes + web profile</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="12" t="n">
+      <c r="A124" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="B124" s="12" t="inlineStr">
+      <c r="B124" s="10" t="inlineStr">
         <is>
           <t>2026-06-26 15:53</t>
         </is>
       </c>
-      <c r="C124" s="12" t="inlineStr">
-        <is>
-          <t>ruby-trivia</t>
-        </is>
-      </c>
-      <c r="D124" s="14" t="inlineStr">
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>ruby-trivia</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
         <is>
           <t>docs(web3): branch for tokenomics/NFT work + compliance guardrails</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="12" t="n">
+      <c r="A125" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="B125" s="12" t="inlineStr">
+      <c r="B125" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:04</t>
         </is>
       </c>
-      <c r="C125" s="12" t="inlineStr">
+      <c r="C125" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D125" s="14" t="inlineStr">
+      <c r="D125" s="12" t="inlineStr">
         <is>
           <t>Add 06: business-structure &amp; governance scaffold (Delaware umbrella, parallel web2/web3, risk-parity control)</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="12" t="n">
+      <c r="A126" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="B126" s="12" t="inlineStr">
+      <c r="B126" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:10</t>
         </is>
       </c>
-      <c r="C126" s="12" t="inlineStr">
+      <c r="C126" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D126" s="14" t="inlineStr">
+      <c r="D126" s="12" t="inlineStr">
         <is>
           <t>Add 07: tax &amp; legal/regulatory research (cited) for the governance structure</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="12" t="n">
+      <c r="A127" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="B127" s="12" t="inlineStr">
+      <c r="B127" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 19:17</t>
         </is>
       </c>
-      <c r="C127" s="12" t="inlineStr">
+      <c r="C127" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D127" s="14" t="inlineStr">
+      <c r="D127" s="12" t="inlineStr">
         <is>
           <t>Add 08: latest 2025-26 statutes + how-others-do-it playbooks + right-sized recommended path</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="12" t="n">
+      <c r="A128" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="B128" s="12" t="inlineStr">
+      <c r="B128" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:05</t>
         </is>
       </c>
-      <c r="C128" s="12" t="inlineStr">
+      <c r="C128" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D128" s="14" t="inlineStr">
+      <c r="D128" s="12" t="inlineStr">
         <is>
           <t>Add browsable docs hub (README front page) + S-corp analysis across 06/07/08</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="12" t="n">
+      <c r="A129" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="B129" s="12" t="inlineStr">
+      <c r="B129" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:22</t>
         </is>
       </c>
-      <c r="C129" s="12" t="inlineStr">
+      <c r="C129" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D129" s="14" t="inlineStr">
+      <c r="D129" s="12" t="inlineStr">
         <is>
           <t>Add founder/operator compensation working proposal (24h counter window) to 06; thread through 07/08/README</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="12" t="n">
+      <c r="A130" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="B130" s="12" t="inlineStr">
+      <c r="B130" s="10" t="inlineStr">
         <is>
           <t>2026-06-29 20:50</t>
         </is>
       </c>
-      <c r="C130" s="12" t="inlineStr">
+      <c r="C130" s="10" t="inlineStr">
         <is>
           <t>ruby-marketing</t>
         </is>
       </c>
-      <c r="D130" s="14" t="inlineStr">
+      <c r="D130" s="12" t="inlineStr">
         <is>
           <t>Comp: operator draw is CAPPED at a fair daily wage (excess stays in treasury)</t>
         </is>
@@ -3888,28 +3872,28 @@
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>• Hours from GitHub commit timestamps. Floor = git-hours method (&gt;2h gap=new session, +2h ramp). Realistic = active-day method weighted by commit intensity (heaviest day ~16h, normal active day ~8h).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>• All commits under 'dutch &lt;dutchiono@gmail.com&gt;' / GitHub 'dutchiono' across all Ruby repos. Other contributors excluded.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>• Date range 2026-05-29 to 2026-06-29; 13 active days; 127 commits.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>• Amount paid to date: $350. Three rate scenarios: $10, $50, $150/hr.</t>
         </is>

</xml_diff>

<commit_message>
Document it all: agreed deal (6/18) + work + pay + dated walk-back, on the page; evidence sheets in workbook
</commit_message>
<xml_diff>
--- a/Dutch-Ruby-Comp-Claim.xlsx
+++ b/Dutch-Ruby-Comp-Claim.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What was built" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commit Log" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Agreement" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Walk-Back" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3902,4 +3904,379 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The deal — agreed and pinned, June 18 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Quote (verbatim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Odi (pinned)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>split of launch generated token allocation (dev fees + agent fees): 50% goes into the dev fund and then we have you down for 7.5% of the total generated in the first week. The 7.5% is for all the work you've done so far. Fees after the first week will go into the dev fund. And then when we have funds we will contract with you for work, full hourly rate, we pay for work done. Happy to even pay 50% upfront. We do not have you down for any equity in the company. If that's something you're interested in, we can talk about it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>btw what is your hour rate for ruby work after launch?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>lets say $50/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>That would be pretty damn comfortable for me for a long time</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Fair is fair and I'm sure it is</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Jun 18 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>I built a whole game and hopefully we get that launched bc I get dev fees</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How the terms were walked back, June 29-30 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Quote (verbatim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 10:59 PM</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>I made $50 for the last three weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:00 PM</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>6.7k, or even half that, and then $50 an hour after ... That was the deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:04 PM</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>what I wrote above it more than $50, however it ain't $5k either</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:06 PM</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>My contract however is fulfilled on my side and currently unpaid</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 10:51 PM</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>split all revenues 50/50 between Iono and Magic ... Iono should get a cut because we owe him so much</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:22 PM</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Dutch / Odi</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Everyone knows I am owed more  /  hence the terms I drew up above</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:35 PM</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>You can't make me work for free anymore</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 11:38 PM</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>the hard reality is we have nothing to offer you to continue working on the project. There's just no closing that gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 ~9:25 PM</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>no that was never offered or said, 7.5% was the initial ... contingent upon a 3mcap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 ~9:35 PM</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>we do split of money made, this did not make a lot of money, so $5k is way out in left field</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Jun 29 ~9:36 PM</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Odi</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>like is there even enough penciled down to negotiate with</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Pay: $350 = what I took; $50 = their valuation (47c/hr); workbook matches
</commit_message>
<xml_diff>
--- a/Dutch-Ruby-Comp-Claim.xlsx
+++ b/Dutch-Ruby-Comp-Claim.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Amount paid to date</t>
+          <t>Amount I drew from the dev wallet</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -553,103 +553,121 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Effective rate paid ( paid ÷ hours )</t>
-        </is>
+      <c r="A9">
+        <f> effective rate for my work ( $350 ÷ hours )</f>
+        <v/>
       </c>
       <c r="B9" s="5" t="n">
         <v>3.30188679245283</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Their valuation of all the work</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>50</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11">
+        <f> the rate they're offering ( $50 ÷ hours )</f>
+        <v/>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0.4716981132075472</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>The hours at three rates (minus $350 paid):</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Owed</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>$10/hr</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>106</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>1060</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>350</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>$25/hr</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>106</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>2650</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>350</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>2300</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>$50/hr</t>
+          <t>$10/hr</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
         <v>106</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>5300</v>
+        <v>1060</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>350</v>
       </c>
       <c r="E15" s="9" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>$25/hr</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>106</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>2650</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>$50/hr</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>106</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>5300</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="E17" s="9" t="n">
         <v>4950</v>
       </c>
     </row>

</xml_diff>